<commit_message>
Updates for adding Chroma DB
</commit_message>
<xml_diff>
--- a/reports/batch_resume_model_comparison.xlsx
+++ b/reports/batch_resume_model_comparison.xlsx
@@ -516,7 +516,7 @@
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>0.0706</v>
+        <v>0.0897</v>
       </c>
     </row>
     <row r="3">
@@ -536,13 +536,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.7381</v>
+        <v>0.7621</v>
       </c>
       <c r="E3" t="n">
         <v>0.4091</v>
       </c>
       <c r="F3" t="n">
-        <v>0.6394</v>
+        <v>0.6562</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -561,7 +561,7 @@
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="n">
-        <v>0.118</v>
+        <v>0.0954</v>
       </c>
     </row>
     <row r="4">
@@ -606,7 +606,7 @@
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="n">
-        <v>0.0591</v>
+        <v>0.0969</v>
       </c>
     </row>
     <row r="5">
@@ -651,7 +651,7 @@
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="n">
-        <v>0.0733</v>
+        <v>0.0397</v>
       </c>
     </row>
     <row r="6">
@@ -671,13 +671,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.7696</v>
+        <v>0.8022</v>
       </c>
       <c r="E6" t="n">
         <v>0.4375</v>
       </c>
       <c r="F6" t="n">
-        <v>0.67</v>
+        <v>0.6928</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -696,7 +696,7 @@
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="n">
-        <v>0.0419</v>
+        <v>0.0389</v>
       </c>
     </row>
     <row r="7">
@@ -741,7 +741,7 @@
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="n">
-        <v>0.0403</v>
+        <v>0.0458</v>
       </c>
     </row>
     <row r="8">
@@ -786,7 +786,7 @@
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="n">
-        <v>0.0808</v>
+        <v>0.0317</v>
       </c>
     </row>
     <row r="9">
@@ -806,13 +806,13 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.6434</v>
+        <v>0.6385999999999999</v>
       </c>
       <c r="E9" t="n">
         <v>0.8333</v>
       </c>
       <c r="F9" t="n">
-        <v>0.7004</v>
+        <v>0.697</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -831,7 +831,7 @@
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="n">
-        <v>0.0318</v>
+        <v>0.0315</v>
       </c>
     </row>
     <row r="10">
@@ -876,7 +876,7 @@
       </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="n">
-        <v>0.0393</v>
+        <v>0.0379</v>
       </c>
     </row>
     <row r="11">
@@ -921,7 +921,7 @@
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="n">
-        <v>0.0663</v>
+        <v>0.0333</v>
       </c>
     </row>
     <row r="12">
@@ -941,13 +941,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.6316000000000001</v>
+        <v>0.6303</v>
       </c>
       <c r="E12" t="n">
         <v>0.2941</v>
       </c>
       <c r="F12" t="n">
-        <v>0.5304</v>
+        <v>0.5294</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -966,7 +966,7 @@
       </c>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="n">
-        <v>0.0346</v>
+        <v>0.0335</v>
       </c>
     </row>
     <row r="13">
@@ -1011,7 +1011,7 @@
       </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="n">
-        <v>0.0347</v>
+        <v>0.0405</v>
       </c>
     </row>
     <row r="14">
@@ -1058,7 +1058,7 @@
         <v>1</v>
       </c>
       <c r="K14" t="n">
-        <v>0.0379</v>
+        <v>0.0372</v>
       </c>
     </row>
     <row r="15">
@@ -1078,13 +1078,13 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.8706</v>
+        <v>0.8716</v>
       </c>
       <c r="E15" t="n">
         <v>0.8636</v>
       </c>
       <c r="F15" t="n">
-        <v>0.8685</v>
+        <v>0.8692</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1105,7 +1105,7 @@
         <v>1</v>
       </c>
       <c r="K15" t="n">
-        <v>0.0733</v>
+        <v>0.0369</v>
       </c>
     </row>
     <row r="16">
@@ -1152,7 +1152,7 @@
         <v>1</v>
       </c>
       <c r="K16" t="n">
-        <v>0.0363</v>
+        <v>0.0418</v>
       </c>
     </row>
     <row r="17">
@@ -1199,7 +1199,7 @@
         <v>1</v>
       </c>
       <c r="K17" t="n">
-        <v>0.1009</v>
+        <v>0.036</v>
       </c>
     </row>
     <row r="18">
@@ -1219,13 +1219,13 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.7934</v>
+        <v>0.7819</v>
       </c>
       <c r="E18" t="n">
         <v>0.75</v>
       </c>
       <c r="F18" t="n">
-        <v>0.7804</v>
+        <v>0.7723</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1246,7 +1246,7 @@
         <v>1</v>
       </c>
       <c r="K18" t="n">
-        <v>0.0573</v>
+        <v>0.0367</v>
       </c>
     </row>
     <row r="19">
@@ -1293,7 +1293,7 @@
         <v>1</v>
       </c>
       <c r="K19" t="n">
-        <v>0.0359</v>
+        <v>0.0435</v>
       </c>
     </row>
     <row r="20">
@@ -1340,7 +1340,7 @@
         <v>1</v>
       </c>
       <c r="K20" t="n">
-        <v>0.08450000000000001</v>
+        <v>0.0366</v>
       </c>
     </row>
     <row r="21">
@@ -1360,13 +1360,13 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.6106</v>
+        <v>0.5895</v>
       </c>
       <c r="E21" t="n">
         <v>0.6667</v>
       </c>
       <c r="F21" t="n">
-        <v>0.6274</v>
+        <v>0.6127</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1387,7 +1387,7 @@
         <v>1</v>
       </c>
       <c r="K21" t="n">
-        <v>0.0373</v>
+        <v>0.0376</v>
       </c>
     </row>
     <row r="22">
@@ -1434,7 +1434,7 @@
         <v>1</v>
       </c>
       <c r="K22" t="n">
-        <v>0.0476</v>
+        <v>0.0432</v>
       </c>
     </row>
     <row r="23">
@@ -1481,7 +1481,7 @@
         <v>1</v>
       </c>
       <c r="K23" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.0382</v>
       </c>
     </row>
     <row r="24">
@@ -1501,13 +1501,13 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.7786</v>
+        <v>0.7675999999999999</v>
       </c>
       <c r="E24" t="n">
         <v>0.5881999999999999</v>
       </c>
       <c r="F24" t="n">
-        <v>0.7215</v>
+        <v>0.7138</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -1528,7 +1528,7 @@
         <v>1</v>
       </c>
       <c r="K24" t="n">
-        <v>0.0365</v>
+        <v>0.0378</v>
       </c>
     </row>
     <row r="25">
@@ -1575,7 +1575,7 @@
         <v>1</v>
       </c>
       <c r="K25" t="n">
-        <v>0.049</v>
+        <v>0.0433</v>
       </c>
     </row>
     <row r="26">
@@ -1620,7 +1620,7 @@
       </c>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="n">
-        <v>0.0437</v>
+        <v>0.0446</v>
       </c>
     </row>
     <row r="27">
@@ -1640,13 +1640,13 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.6068</v>
+        <v>0.6218</v>
       </c>
       <c r="E27" t="n">
         <v>0.4091</v>
       </c>
       <c r="F27" t="n">
-        <v>0.5475</v>
+        <v>0.5580000000000001</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -1665,7 +1665,7 @@
       </c>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="n">
-        <v>0.0466</v>
+        <v>0.0429</v>
       </c>
     </row>
     <row r="28">
@@ -1710,7 +1710,7 @@
       </c>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="n">
-        <v>0.074</v>
+        <v>0.0461</v>
       </c>
     </row>
     <row r="29">
@@ -1755,7 +1755,7 @@
       </c>
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="n">
-        <v>0.0445</v>
+        <v>0.0395</v>
       </c>
     </row>
     <row r="30">
@@ -1775,13 +1775,13 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0.5072</v>
+        <v>0.5004</v>
       </c>
       <c r="E30" t="n">
         <v>0.4375</v>
       </c>
       <c r="F30" t="n">
-        <v>0.4863</v>
+        <v>0.4815</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1800,7 +1800,7 @@
       </c>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="n">
-        <v>0.0336</v>
+        <v>0.0418</v>
       </c>
     </row>
     <row r="31">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="n">
-        <v>0.0532</v>
+        <v>0.0492</v>
       </c>
     </row>
     <row r="32">
@@ -1890,7 +1890,7 @@
       </c>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="n">
-        <v>0.0596</v>
+        <v>0.0439</v>
       </c>
     </row>
     <row r="33">
@@ -1910,13 +1910,13 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>0.5106000000000001</v>
+        <v>0.5187</v>
       </c>
       <c r="E33" t="n">
         <v>0.1667</v>
       </c>
       <c r="F33" t="n">
-        <v>0.4074</v>
+        <v>0.4131</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -1935,7 +1935,7 @@
       </c>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="n">
-        <v>0.0331</v>
+        <v>0.0443</v>
       </c>
     </row>
     <row r="34">
@@ -1980,7 +1980,7 @@
       </c>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="n">
-        <v>0.0462</v>
+        <v>0.0504</v>
       </c>
     </row>
     <row r="35">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="n">
-        <v>0.0482</v>
+        <v>0.044</v>
       </c>
     </row>
     <row r="36">
@@ -2045,13 +2045,13 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>0.5352</v>
+        <v>0.5222</v>
       </c>
       <c r="E36" t="n">
         <v>0.4118</v>
       </c>
       <c r="F36" t="n">
-        <v>0.4982</v>
+        <v>0.489</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -2070,7 +2070,7 @@
       </c>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="n">
-        <v>0.0342</v>
+        <v>0.0417</v>
       </c>
     </row>
     <row r="37">
@@ -2115,7 +2115,7 @@
       </c>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="n">
-        <v>0.06809999999999999</v>
+        <v>0.0486</v>
       </c>
     </row>
     <row r="38">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="n">
-        <v>0.041</v>
+        <v>0.0396</v>
       </c>
     </row>
     <row r="39">
@@ -2180,13 +2180,13 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>0.8135</v>
+        <v>0.8258</v>
       </c>
       <c r="E39" t="n">
         <v>0.8182</v>
       </c>
       <c r="F39" t="n">
-        <v>0.8149</v>
+        <v>0.8235</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -2205,7 +2205,7 @@
       </c>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="n">
-        <v>0.035</v>
+        <v>0.0371</v>
       </c>
     </row>
     <row r="40">
@@ -2250,7 +2250,7 @@
       </c>
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="n">
-        <v>0.0356</v>
+        <v>0.0403</v>
       </c>
     </row>
     <row r="41">
@@ -2295,7 +2295,7 @@
       </c>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="n">
-        <v>0.1085</v>
+        <v>0.0348</v>
       </c>
     </row>
     <row r="42">
@@ -2315,13 +2315,13 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>0.8046</v>
+        <v>0.8164</v>
       </c>
       <c r="E42" t="n">
         <v>0.6875</v>
       </c>
       <c r="F42" t="n">
-        <v>0.7694</v>
+        <v>0.7776999999999999</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -2340,7 +2340,7 @@
       </c>
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="n">
-        <v>0.0317</v>
+        <v>0.0346</v>
       </c>
     </row>
     <row r="43">
@@ -2385,7 +2385,7 @@
       </c>
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="n">
-        <v>0.035</v>
+        <v>0.0416</v>
       </c>
     </row>
     <row r="44">
@@ -2426,7 +2426,7 @@
       </c>
       <c r="J44" t="inlineStr"/>
       <c r="K44" t="n">
-        <v>0.09089999999999999</v>
+        <v>0.0382</v>
       </c>
     </row>
     <row r="45">
@@ -2446,13 +2446,13 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>0.6159</v>
+        <v>0.613</v>
       </c>
       <c r="E45" t="n">
         <v>1</v>
       </c>
       <c r="F45" t="n">
-        <v>0.7311</v>
+        <v>0.7291</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="J45" t="inlineStr"/>
       <c r="K45" t="n">
-        <v>0.0279</v>
+        <v>0.0379</v>
       </c>
     </row>
     <row r="46">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="J46" t="inlineStr"/>
       <c r="K46" t="n">
-        <v>0.0314</v>
+        <v>0.0437</v>
       </c>
     </row>
     <row r="47">
@@ -2553,7 +2553,7 @@
       </c>
       <c r="J47" t="inlineStr"/>
       <c r="K47" t="n">
-        <v>0.07580000000000001</v>
+        <v>0.0382</v>
       </c>
     </row>
     <row r="48">
@@ -2573,13 +2573,13 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>0.7077</v>
+        <v>0.699</v>
       </c>
       <c r="E48" t="n">
         <v>0.7059</v>
       </c>
       <c r="F48" t="n">
-        <v>0.7072000000000001</v>
+        <v>0.7010999999999999</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -2598,7 +2598,7 @@
       </c>
       <c r="J48" t="inlineStr"/>
       <c r="K48" t="n">
-        <v>0.0385</v>
+        <v>0.038</v>
       </c>
     </row>
     <row r="49">
@@ -2643,7 +2643,7 @@
       </c>
       <c r="J49" t="inlineStr"/>
       <c r="K49" t="n">
-        <v>0.0518</v>
+        <v>0.0441</v>
       </c>
     </row>
   </sheetData>
@@ -2694,16 +2694,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.6835875</v>
+        <v>0.68506875</v>
       </c>
       <c r="C2" t="n">
         <v>0.59245</v>
       </c>
       <c r="D2" t="n">
-        <v>0.65625</v>
+        <v>0.6572749999999999</v>
       </c>
       <c r="E2" t="n">
-        <v>0.04445625</v>
+        <v>0.0416625</v>
       </c>
     </row>
     <row r="3">
@@ -2722,7 +2722,7 @@
         <v>0.566075</v>
       </c>
       <c r="E3" t="n">
-        <v>0.06846874999999999</v>
+        <v>0.041575</v>
       </c>
     </row>
     <row r="4">
@@ -2741,7 +2741,7 @@
         <v>0.566075</v>
       </c>
       <c r="E4" t="n">
-        <v>0.04609375</v>
+        <v>0.04730625</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Changes for relative imports for report related scripts
All scripts are in the ml sub-directory and hence the command to invoke them has to use format, `python -m ml.script_name`
</commit_message>
<xml_diff>
--- a/reports/batch_resume_model_comparison.xlsx
+++ b/reports/batch_resume_model_comparison.xlsx
@@ -516,7 +516,7 @@
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>0.0897</v>
+        <v>0.1209</v>
       </c>
     </row>
     <row r="3">
@@ -561,7 +561,7 @@
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="n">
-        <v>0.0954</v>
+        <v>0.1154</v>
       </c>
     </row>
     <row r="4">
@@ -606,7 +606,7 @@
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="n">
-        <v>0.0969</v>
+        <v>0.0693</v>
       </c>
     </row>
     <row r="5">
@@ -651,7 +651,7 @@
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="n">
-        <v>0.0397</v>
+        <v>0.036</v>
       </c>
     </row>
     <row r="6">
@@ -696,7 +696,7 @@
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="n">
-        <v>0.0389</v>
+        <v>0.0694</v>
       </c>
     </row>
     <row r="7">
@@ -741,7 +741,7 @@
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="n">
-        <v>0.0458</v>
+        <v>0.0615</v>
       </c>
     </row>
     <row r="8">
@@ -786,7 +786,7 @@
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="n">
-        <v>0.0317</v>
+        <v>0.0241</v>
       </c>
     </row>
     <row r="9">
@@ -831,7 +831,7 @@
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="n">
-        <v>0.0315</v>
+        <v>0.0262</v>
       </c>
     </row>
     <row r="10">
@@ -876,7 +876,7 @@
       </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="n">
-        <v>0.0379</v>
+        <v>0.0539</v>
       </c>
     </row>
     <row r="11">
@@ -921,7 +921,7 @@
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="n">
-        <v>0.0333</v>
+        <v>0.0567</v>
       </c>
     </row>
     <row r="12">
@@ -966,7 +966,7 @@
       </c>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="n">
-        <v>0.0335</v>
+        <v>0.0313</v>
       </c>
     </row>
     <row r="13">
@@ -1011,7 +1011,7 @@
       </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="n">
-        <v>0.0405</v>
+        <v>0.0344</v>
       </c>
     </row>
     <row r="14">
@@ -1058,7 +1058,7 @@
         <v>1</v>
       </c>
       <c r="K14" t="n">
-        <v>0.0372</v>
+        <v>0.0696</v>
       </c>
     </row>
     <row r="15">
@@ -1105,7 +1105,7 @@
         <v>1</v>
       </c>
       <c r="K15" t="n">
-        <v>0.0369</v>
+        <v>0.041</v>
       </c>
     </row>
     <row r="16">
@@ -1152,7 +1152,7 @@
         <v>1</v>
       </c>
       <c r="K16" t="n">
-        <v>0.0418</v>
+        <v>0.0307</v>
       </c>
     </row>
     <row r="17">
@@ -1199,7 +1199,7 @@
         <v>1</v>
       </c>
       <c r="K17" t="n">
-        <v>0.036</v>
+        <v>0.0847</v>
       </c>
     </row>
     <row r="18">
@@ -1246,7 +1246,7 @@
         <v>1</v>
       </c>
       <c r="K18" t="n">
-        <v>0.0367</v>
+        <v>0.0443</v>
       </c>
     </row>
     <row r="19">
@@ -1293,7 +1293,7 @@
         <v>1</v>
       </c>
       <c r="K19" t="n">
-        <v>0.0435</v>
+        <v>0.0356</v>
       </c>
     </row>
     <row r="20">
@@ -1340,7 +1340,7 @@
         <v>1</v>
       </c>
       <c r="K20" t="n">
-        <v>0.0366</v>
+        <v>0.08690000000000001</v>
       </c>
     </row>
     <row r="21">
@@ -1387,7 +1387,7 @@
         <v>1</v>
       </c>
       <c r="K21" t="n">
-        <v>0.0376</v>
+        <v>0.0454</v>
       </c>
     </row>
     <row r="22">
@@ -1434,7 +1434,7 @@
         <v>1</v>
       </c>
       <c r="K22" t="n">
-        <v>0.0432</v>
+        <v>0.0345</v>
       </c>
     </row>
     <row r="23">
@@ -1481,7 +1481,7 @@
         <v>1</v>
       </c>
       <c r="K23" t="n">
-        <v>0.0382</v>
+        <v>0.0871</v>
       </c>
     </row>
     <row r="24">
@@ -1528,7 +1528,7 @@
         <v>1</v>
       </c>
       <c r="K24" t="n">
-        <v>0.0378</v>
+        <v>0.0445</v>
       </c>
     </row>
     <row r="25">
@@ -1575,7 +1575,7 @@
         <v>1</v>
       </c>
       <c r="K25" t="n">
-        <v>0.0433</v>
+        <v>0.0294</v>
       </c>
     </row>
     <row r="26">
@@ -1620,7 +1620,7 @@
       </c>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="n">
-        <v>0.0446</v>
+        <v>0.0572</v>
       </c>
     </row>
     <row r="27">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="n">
-        <v>0.0429</v>
+        <v>0.0331</v>
       </c>
     </row>
     <row r="28">
@@ -1710,7 +1710,7 @@
       </c>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="n">
-        <v>0.0461</v>
+        <v>0.0601</v>
       </c>
     </row>
     <row r="29">
@@ -1755,7 +1755,7 @@
       </c>
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="n">
-        <v>0.0395</v>
+        <v>0.0564</v>
       </c>
     </row>
     <row r="30">
@@ -1800,7 +1800,7 @@
       </c>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="n">
-        <v>0.0418</v>
+        <v>0.0321</v>
       </c>
     </row>
     <row r="31">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="n">
-        <v>0.0492</v>
+        <v>0.0626</v>
       </c>
     </row>
     <row r="32">
@@ -1890,7 +1890,7 @@
       </c>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="n">
-        <v>0.0439</v>
+        <v>0.056</v>
       </c>
     </row>
     <row r="33">
@@ -1935,7 +1935,7 @@
       </c>
       <c r="J33" t="inlineStr"/>
       <c r="K33" t="n">
-        <v>0.0443</v>
+        <v>0.032</v>
       </c>
     </row>
     <row r="34">
@@ -1980,7 +1980,7 @@
       </c>
       <c r="J34" t="inlineStr"/>
       <c r="K34" t="n">
-        <v>0.0504</v>
+        <v>0.0581</v>
       </c>
     </row>
     <row r="35">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="n">
-        <v>0.044</v>
+        <v>0.066</v>
       </c>
     </row>
     <row r="36">
@@ -2070,7 +2070,7 @@
       </c>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="n">
-        <v>0.0417</v>
+        <v>0.0365</v>
       </c>
     </row>
     <row r="37">
@@ -2115,7 +2115,7 @@
       </c>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="n">
-        <v>0.0486</v>
+        <v>0.0446</v>
       </c>
     </row>
     <row r="38">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="n">
-        <v>0.0396</v>
+        <v>0.0519</v>
       </c>
     </row>
     <row r="39">
@@ -2205,7 +2205,7 @@
       </c>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="n">
-        <v>0.0371</v>
+        <v>0.0356</v>
       </c>
     </row>
     <row r="40">
@@ -2250,7 +2250,7 @@
       </c>
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="n">
-        <v>0.0403</v>
+        <v>0.0307</v>
       </c>
     </row>
     <row r="41">
@@ -2295,7 +2295,7 @@
       </c>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="n">
-        <v>0.0348</v>
+        <v>0.1308</v>
       </c>
     </row>
     <row r="42">
@@ -2340,7 +2340,7 @@
       </c>
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="n">
-        <v>0.0346</v>
+        <v>0.0362</v>
       </c>
     </row>
     <row r="43">
@@ -2385,7 +2385,7 @@
       </c>
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="n">
-        <v>0.0416</v>
+        <v>0.0313</v>
       </c>
     </row>
     <row r="44">
@@ -2426,7 +2426,7 @@
       </c>
       <c r="J44" t="inlineStr"/>
       <c r="K44" t="n">
-        <v>0.0382</v>
+        <v>0.0677</v>
       </c>
     </row>
     <row r="45">
@@ -2467,7 +2467,7 @@
       </c>
       <c r="J45" t="inlineStr"/>
       <c r="K45" t="n">
-        <v>0.0379</v>
+        <v>0.0443</v>
       </c>
     </row>
     <row r="46">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="J46" t="inlineStr"/>
       <c r="K46" t="n">
-        <v>0.0437</v>
+        <v>0.0396</v>
       </c>
     </row>
     <row r="47">
@@ -2553,7 +2553,7 @@
       </c>
       <c r="J47" t="inlineStr"/>
       <c r="K47" t="n">
-        <v>0.0382</v>
+        <v>0.1316</v>
       </c>
     </row>
     <row r="48">
@@ -2598,7 +2598,7 @@
       </c>
       <c r="J48" t="inlineStr"/>
       <c r="K48" t="n">
-        <v>0.038</v>
+        <v>0.0316</v>
       </c>
     </row>
     <row r="49">
@@ -2643,7 +2643,7 @@
       </c>
       <c r="J49" t="inlineStr"/>
       <c r="K49" t="n">
-        <v>0.0441</v>
+        <v>0.0313</v>
       </c>
     </row>
   </sheetData>
@@ -2703,7 +2703,7 @@
         <v>0.6572749999999999</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0416625</v>
+        <v>0.04368125</v>
       </c>
     </row>
     <row r="3">
@@ -2722,7 +2722,7 @@
         <v>0.566075</v>
       </c>
       <c r="E3" t="n">
-        <v>0.041575</v>
+        <v>0.073975</v>
       </c>
     </row>
     <row r="4">
@@ -2741,7 +2741,7 @@
         <v>0.566075</v>
       </c>
       <c r="E4" t="n">
-        <v>0.04730625</v>
+        <v>0.044225</v>
       </c>
     </row>
   </sheetData>

</xml_diff>